<commit_message>
Fix UI/UX issues for bottom tab on web and complete E2E testing fixes
</commit_message>
<xml_diff>
--- a/automated_test/selenium_report.xlsx
+++ b/automated_test/selenium_report.xlsx
@@ -43,7 +43,7 @@
     <t>Successfully loaded http://localhost:8081 and cleared state</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:29.064Z</t>
+    <t>2026-06-16T14:03:59.152Z</t>
   </si>
   <si>
     <t>TC-02</t>
@@ -55,7 +55,7 @@
     <t>Routed to Login page correctly: http://localhost:8081/login</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:32.232Z</t>
+    <t>2026-06-16T14:04:02.393Z</t>
   </si>
   <si>
     <t>TC-03</t>
@@ -67,7 +67,7 @@
     <t>Found 2 input field(s).</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:32.260Z</t>
+    <t>2026-06-16T14:04:02.435Z</t>
   </si>
   <si>
     <t>TC-04</t>
@@ -79,7 +79,7 @@
     <t xml:space="preserve">Received correct failure notification: </t>
   </si>
   <si>
-    <t>2026-06-14T13:22:33.844Z</t>
+    <t>2026-06-16T14:04:04.331Z</t>
   </si>
   <si>
     <t>TC-05</t>
@@ -91,7 +91,7 @@
     <t>Authenticated successfully with Sanjay29 profile</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:35.249Z</t>
+    <t>2026-06-16T14:04:05.997Z</t>
   </si>
   <si>
     <t>TC-06</t>
@@ -103,7 +103,7 @@
     <t>Dashboard header and options rendered successfully.</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:35.259Z</t>
+    <t>2026-06-16T14:04:06.010Z</t>
   </si>
   <si>
     <t>TC-07</t>
@@ -115,7 +115,7 @@
     <t>Successfully routed to upload page for Rental Agreement.</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:35.355Z</t>
+    <t>2026-06-16T14:04:06.151Z</t>
   </si>
   <si>
     <t>TC-08</t>
@@ -127,7 +127,7 @@
     <t>Successfully selected mock dummy.jpg document</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:35.552Z</t>
+    <t>2026-06-16T14:04:06.360Z</t>
   </si>
   <si>
     <t>TC-09</t>
@@ -139,7 +139,7 @@
     <t>Audit completed successfully! Routed to: http://localhost:8081/results?category=rental&amp;result=%7B%22parsed%22%3A%7B%22vendor%22%3A%22HSR%20Apartment%204B%22%2C%22date%22%3A%22Jun%2014%2C%202026%22%2C%22subtotal%22%3A%2218000%22%2C%22tax%22%3A%220%22%2C%22total%22%3A%2218000%22%7D%2C%22all_details%22%3A%5B%7B%22label%22%3A%22Vendor%20Name%22%2C%22value%22%3A%22HSR%20Apartment%204B%22%7D%2C%7B%22label%22%3A%22Invoice%20Date%22%2C%22value%22%3A%22Jun%2014%2C%202026%22%7D%2C%7B%22label%22%3A%22Rent%20Amount%22%2C%22value%22%3A%22%E2%82%B918%2C000%22%7D%5D%2C%22verdict%22%3A%22overcharged%22%2C%22savings%22%3A1500%2C%22findings%22%3A%5B%7B%22status%22%3A%22error%22%2C%22label%22%3A%22Base%20rent%20mismatch%22%2C%22delta%22%3A%22%E2%82%B91%2C500%22%7D%5D%2C%22recommendation%22%3A%22Overcharged%20detected%22%2C%22message%22%3A%22Overcharged%20detected%22%7D</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:36.507Z</t>
+    <t>2026-06-16T14:04:07.332Z</t>
   </si>
   <si>
     <t>TC-10</t>
@@ -151,7 +151,7 @@
     <t>Successfully verified user session remains logged in after page refresh</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:39.989Z</t>
+    <t>2026-06-16T14:04:09.795Z</t>
   </si>
   <si>
     <t>TC-11</t>
@@ -163,7 +163,7 @@
     <t>Successfully navigated to profile page and signed out of session</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:43.085Z</t>
+    <t>2026-06-16T14:04:12.119Z</t>
   </si>
   <si>
     <t>TC-12</t>
@@ -175,7 +175,7 @@
     <t>Successfully registered new user selenium_tester and logged in</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:45.919Z</t>
+    <t>2026-06-16T14:04:14.935Z</t>
   </si>
   <si>
     <t>TC-13</t>
@@ -187,7 +187,7 @@
     <t>Session persists for dynamically registered custom accounts</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:50.307Z</t>
+    <t>2026-06-16T14:04:18.832Z</t>
   </si>
   <si>
     <t>TC-14</t>
@@ -199,7 +199,7 @@
     <t>Successfully logged in dynamically via Google SSO with mail prefix profile</t>
   </si>
   <si>
-    <t>2026-06-14T13:22:58.212Z</t>
+    <t>2026-06-16T14:04:25.773Z</t>
   </si>
   <si>
     <t>TC-15</t>
@@ -211,7 +211,7 @@
     <t>Google SSO authenticated session successfully persists across browser reloads</t>
   </si>
   <si>
-    <t>2026-06-14T13:23:02.733Z</t>
+    <t>2026-06-16T14:04:29.732Z</t>
   </si>
 </sst>
 </file>
@@ -652,7 +652,7 @@
         <v>8</v>
       </c>
       <c r="D2">
-        <v>5726</v>
+        <v>11735</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
@@ -672,7 +672,7 @@
         <v>8</v>
       </c>
       <c r="D3">
-        <v>3154</v>
+        <v>3230</v>
       </c>
       <c r="E3" t="s">
         <v>13</v>
@@ -692,7 +692,7 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
         <v>17</v>
@@ -712,7 +712,7 @@
         <v>8</v>
       </c>
       <c r="D5">
-        <v>1583</v>
+        <v>1895</v>
       </c>
       <c r="E5" t="s">
         <v>21</v>
@@ -732,7 +732,7 @@
         <v>8</v>
       </c>
       <c r="D6">
-        <v>1405</v>
+        <v>1666</v>
       </c>
       <c r="E6" t="s">
         <v>25</v>
@@ -752,7 +752,7 @@
         <v>8</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
         <v>29</v>
@@ -772,7 +772,7 @@
         <v>8</v>
       </c>
       <c r="D8">
-        <v>96</v>
+        <v>141</v>
       </c>
       <c r="E8" t="s">
         <v>33</v>
@@ -792,7 +792,7 @@
         <v>8</v>
       </c>
       <c r="D9">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="E9" t="s">
         <v>37</v>
@@ -812,7 +812,7 @@
         <v>8</v>
       </c>
       <c r="D10">
-        <v>946</v>
+        <v>949</v>
       </c>
       <c r="E10" t="s">
         <v>41</v>
@@ -832,7 +832,7 @@
         <v>8</v>
       </c>
       <c r="D11">
-        <v>3482</v>
+        <v>2463</v>
       </c>
       <c r="E11" t="s">
         <v>45</v>
@@ -852,7 +852,7 @@
         <v>8</v>
       </c>
       <c r="D12">
-        <v>3096</v>
+        <v>2324</v>
       </c>
       <c r="E12" t="s">
         <v>49</v>
@@ -872,7 +872,7 @@
         <v>8</v>
       </c>
       <c r="D13">
-        <v>2834</v>
+        <v>2816</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -892,7 +892,7 @@
         <v>8</v>
       </c>
       <c r="D14">
-        <v>4388</v>
+        <v>3896</v>
       </c>
       <c r="E14" t="s">
         <v>57</v>
@@ -912,7 +912,7 @@
         <v>8</v>
       </c>
       <c r="D15">
-        <v>7905</v>
+        <v>6941</v>
       </c>
       <c r="E15" t="s">
         <v>61</v>
@@ -932,7 +932,7 @@
         <v>8</v>
       </c>
       <c r="D16">
-        <v>4520</v>
+        <v>3959</v>
       </c>
       <c r="E16" t="s">
         <v>65</v>

</xml_diff>